<commit_message>
Updated error handler and order processing
</commit_message>
<xml_diff>
--- a/Processed_Orders_by_DC.xlsx
+++ b/Processed_Orders_by_DC.xlsx
@@ -10,13 +10,15 @@
     <sheet name="DC01" sheetId="1" r:id="rId1"/>
     <sheet name="DC02" sheetId="2" r:id="rId2"/>
     <sheet name="DC03" sheetId="3" r:id="rId3"/>
+    <sheet name="DC04" sheetId="4" r:id="rId4"/>
+    <sheet name="DC05" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="24">
   <si>
     <t>OrderID</t>
   </si>
@@ -30,6 +32,9 @@
     <t>OrderDate</t>
   </si>
   <si>
+    <t>ProcessingRule</t>
+  </si>
+  <si>
     <t>ORD001</t>
   </si>
   <si>
@@ -42,6 +47,9 @@
     <t>2024-01-10</t>
   </si>
   <si>
+    <t>Ready for invoicing</t>
+  </si>
+  <si>
     <t>ORD002</t>
   </si>
   <si>
@@ -54,6 +62,9 @@
     <t>2024-01-11</t>
   </si>
   <si>
+    <t>Pending verification</t>
+  </si>
+  <si>
     <t>ORD003</t>
   </si>
   <si>
@@ -61,6 +72,24 @@
   </si>
   <si>
     <t>2024-01-12</t>
+  </si>
+  <si>
+    <t>ORD005</t>
+  </si>
+  <si>
+    <t>DC04</t>
+  </si>
+  <si>
+    <t>2024-01-14 00:00:00</t>
+  </si>
+  <si>
+    <t>ORD006</t>
+  </si>
+  <si>
+    <t>DC05</t>
+  </si>
+  <si>
+    <t>Missing status code</t>
   </si>
 </sst>
 </file>
@@ -418,10 +447,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -434,19 +463,25 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -456,10 +491,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -472,19 +507,25 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>13</v>
+      </c>
+      <c r="E2" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -494,10 +535,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -510,19 +551,110 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" t="s">
         <v>12</v>
       </c>
+      <c r="D2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>21</v>
+      </c>
       <c r="B2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="D2" t="s">
-        <v>14</v>
+        <v>20</v>
+      </c>
+      <c r="E2" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>